<commit_message>
Add total row and polish dashboard
</commit_message>
<xml_diff>
--- a/docs/data/polymarket_30d_topic_share.xlsx
+++ b/docs/data/polymarket_30d_topic_share.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="current" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="history" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="current" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="history" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,8 +30,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +44,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002D5A87"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF2F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,13 +64,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -631,6 +642,27 @@
       </c>
       <c r="E9" t="n">
         <v>7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>18607918511.16997</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>2000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>